<commit_message>
feat: add sample Excel file for student imports
</commit_message>
<xml_diff>
--- a/public/samples/import_student_sample.xlsx
+++ b/public/samples/import_student_sample.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="31">
   <si>
     <t>ULTRA ENGLISH SCHOOL       1-A</t>
   </si>
@@ -45,148 +45,28 @@
     <t>RELIGION</t>
   </si>
   <si>
-    <t>BALAS DHIYA DINESHBHAI</t>
-  </si>
-  <si>
-    <t>2502</t>
-  </si>
-  <si>
-    <t>9409448248</t>
-  </si>
-  <si>
-    <t>16-03-20</t>
-  </si>
-  <si>
-    <t>06-05-2026</t>
-  </si>
-  <si>
-    <t>CHAMPABEN</t>
-  </si>
-  <si>
-    <t>KOLI (GHEDIYA)</t>
+    <t>PATEL AARAV RAMESHBHAI</t>
+  </si>
+  <si>
+    <t>1001</t>
+  </si>
+  <si>
+    <t>9876543210</t>
+  </si>
+  <si>
+    <t>15-05-2018</t>
+  </si>
+  <si>
+    <t>01-06-2024</t>
+  </si>
+  <si>
+    <t>GITABEN</t>
+  </si>
+  <si>
+    <t>PATEL</t>
   </si>
   <si>
     <t>Hindu</t>
-  </si>
-  <si>
-    <t>DHADUK ANSHI SAMIRBHAI</t>
-  </si>
-  <si>
-    <t>2506</t>
-  </si>
-  <si>
-    <t>9712576222</t>
-  </si>
-  <si>
-    <t>23-04-20</t>
-  </si>
-  <si>
-    <t>06-06-2026</t>
-  </si>
-  <si>
-    <t>BHUMIKABEN</t>
-  </si>
-  <si>
-    <t>LEUVA PATEL</t>
-  </si>
-  <si>
-    <t>SETA PRINCESS JITENKUMAR</t>
-  </si>
-  <si>
-    <t>2488</t>
-  </si>
-  <si>
-    <t>8200399722</t>
-  </si>
-  <si>
-    <t>05-08-19</t>
-  </si>
-  <si>
-    <t>01-07-2025</t>
-  </si>
-  <si>
-    <t>POOJABEN</t>
-  </si>
-  <si>
-    <t>LOHANA</t>
-  </si>
-  <si>
-    <t>BUDHANI AARUSH SANJAY</t>
-  </si>
-  <si>
-    <t>2507</t>
-  </si>
-  <si>
-    <t>6351247064</t>
-  </si>
-  <si>
-    <t>04-01-20</t>
-  </si>
-  <si>
-    <t>HINA</t>
-  </si>
-  <si>
-    <t>SINDHI</t>
-  </si>
-  <si>
-    <t>JADAV JAY PRAFULBHAI</t>
-  </si>
-  <si>
-    <t>2503</t>
-  </si>
-  <si>
-    <t>9662913520</t>
-  </si>
-  <si>
-    <t>22-06-19</t>
-  </si>
-  <si>
-    <t>08-05-2026</t>
-  </si>
-  <si>
-    <t>MANISHABEN</t>
-  </si>
-  <si>
-    <t>VANKAR</t>
-  </si>
-  <si>
-    <t>MEGHAPARA DARSH KETANBHAI</t>
-  </si>
-  <si>
-    <t>2484</t>
-  </si>
-  <si>
-    <t>9913104918</t>
-  </si>
-  <si>
-    <t>16-09-19</t>
-  </si>
-  <si>
-    <t>11-06-2025</t>
-  </si>
-  <si>
-    <t>RANJUBEN</t>
-  </si>
-  <si>
-    <t>KADVA KANABI</t>
-  </si>
-  <si>
-    <t>VARU KRISHIV MANISHBHAI</t>
-  </si>
-  <si>
-    <t>2504</t>
-  </si>
-  <si>
-    <t>9722313334</t>
-  </si>
-  <si>
-    <t>19-10-19</t>
-  </si>
-  <si>
-    <t>JAYNABEN</t>
-  </si>
-  <si>
-    <t>PRAJAPATI</t>
   </si>
   <si>
     <t>HOW TO PREPARE THE IMPORT FILE</t>
@@ -591,7 +471,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="30.564" customWidth="true" style="0"/>
@@ -608,6 +488,7 @@
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="H1"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="1" t="s">
@@ -658,162 +539,6 @@
         <v>15</v>
       </c>
       <c r="H3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" t="s">
-        <v>22</v>
-      </c>
-      <c r="G4" t="s">
-        <v>23</v>
-      </c>
-      <c r="H4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B5" t="s">
-        <v>25</v>
-      </c>
-      <c r="C5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D5" t="s">
-        <v>27</v>
-      </c>
-      <c r="E5" t="s">
-        <v>28</v>
-      </c>
-      <c r="F5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G5" t="s">
-        <v>30</v>
-      </c>
-      <c r="H5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
-      <c r="A6" t="s">
-        <v>31</v>
-      </c>
-      <c r="B6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C6" t="s">
-        <v>33</v>
-      </c>
-      <c r="D6" t="s">
-        <v>34</v>
-      </c>
-      <c r="E6" t="s">
-        <v>21</v>
-      </c>
-      <c r="F6" t="s">
-        <v>35</v>
-      </c>
-      <c r="G6" t="s">
-        <v>36</v>
-      </c>
-      <c r="H6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8">
-      <c r="A7" t="s">
-        <v>37</v>
-      </c>
-      <c r="B7" t="s">
-        <v>38</v>
-      </c>
-      <c r="C7" t="s">
-        <v>39</v>
-      </c>
-      <c r="D7" t="s">
-        <v>40</v>
-      </c>
-      <c r="E7" t="s">
-        <v>41</v>
-      </c>
-      <c r="F7" t="s">
-        <v>42</v>
-      </c>
-      <c r="G7" t="s">
-        <v>43</v>
-      </c>
-      <c r="H7" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
-      <c r="A8" t="s">
-        <v>44</v>
-      </c>
-      <c r="B8" t="s">
-        <v>45</v>
-      </c>
-      <c r="C8" t="s">
-        <v>46</v>
-      </c>
-      <c r="D8" t="s">
-        <v>47</v>
-      </c>
-      <c r="E8" t="s">
-        <v>48</v>
-      </c>
-      <c r="F8" t="s">
-        <v>49</v>
-      </c>
-      <c r="G8" t="s">
-        <v>50</v>
-      </c>
-      <c r="H8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8">
-      <c r="A9" t="s">
-        <v>51</v>
-      </c>
-      <c r="B9" t="s">
-        <v>52</v>
-      </c>
-      <c r="C9" t="s">
-        <v>53</v>
-      </c>
-      <c r="D9" t="s">
-        <v>54</v>
-      </c>
-      <c r="E9" t="s">
-        <v>41</v>
-      </c>
-      <c r="F9" t="s">
-        <v>55</v>
-      </c>
-      <c r="G9" t="s">
-        <v>56</v>
-      </c>
-      <c r="H9" t="s">
         <v>16</v>
       </c>
     </row>
@@ -849,7 +574,7 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="3" t="s">
-        <v>57</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:1">
@@ -857,62 +582,62 @@
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>59</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>60</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>61</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" t="s">
-        <v>62</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" t="s">
-        <v>63</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" t="s">
-        <v>64</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" t="s">
-        <v>65</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" t="s">
-        <v>66</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" t="s">
-        <v>67</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:1">
       <c r="A13" t="s">
-        <v>68</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14" spans="1:1">
       <c r="A14" t="s">
-        <v>69</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" spans="1:1">
@@ -920,7 +645,7 @@
     </row>
     <row r="16" spans="1:1">
       <c r="A16" t="s">
-        <v>70</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>